<commit_message>
docs(sprint3): align test cases, execution log, bug reports, and audit with review
Unify 30 test cases and executions, make failed-to-report mapping strictly one-to-one, correct severity and priority per the method guide, and sync all Sprint 3 documents with the GitHub tracker.
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run 1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run 1'!$A$1:$L$32</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,28 +32,10 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C65911"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00833C0C"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -64,26 +48,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+        <fgColor rgb="000F4C81"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,41 +77,38 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B7C4D1"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B7C4D1"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B7C4D1"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B7C4D1"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -498,22 +475,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Run</t>
@@ -561,7 +540,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Фактичний результат та примітки</t>
+          <t>Крок</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Час</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Коментар</t>
         </is>
       </c>
     </row>
@@ -581,9 +570,9 @@
           <t>F-10, GUI-10</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Успішний вхід студента за валідними логіном та паролем</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Успішний вхід студента з валідними обліковими даними та вихід із системи</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -598,10 +587,10 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -611,9 +600,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Успішна автентифікація. Редірект на /my/. Профіль 'Student User' відображається коректно.</t>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Редірект на /my/; роль і меню відповідають очікуваному; сторінка відкрита через HTTPS.</t>
         </is>
       </c>
     </row>
@@ -633,9 +632,9 @@
           <t>F-10, GUI-20</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Помилка входу при невірному паролі зі збереженням логіну</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Помилка входу з невірним паролем: збереження логіна, очищення пароля, фокус у полі «Пароль»</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -650,22 +649,32 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>BUG-008</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Повідомлення показано, але фокус курсора втрачається з поля пароля (порушення GUI-20).</t>
+          <t>BUG-001</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Повідомлення і збереження логіна збігаються, але фокус залишився на кнопці «Увійти»; символ x у поле пароля не потрапив.</t>
         </is>
       </c>
     </row>
@@ -685,9 +694,9 @@
           <t>F-10, S-20</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Блокування облікового запису на 15 хв після 3 невдалих спроб</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Блокування облікового запису на 15 хвилин після 3 невдалих спроб входу</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -702,22 +711,32 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>BUG-001</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Після 3 невдалих спроб введення блокування акаунту на 15 хв не активується. Вхід за правильним паролем пускає.</t>
+          <t>BUG-002</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Після 3-ї невдалої спроби лічильник показує 0, але блокування немає: вхід із sandbox24 успішний.</t>
         </is>
       </c>
     </row>
@@ -737,9 +756,9 @@
           <t>F-20</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Запит на скидання пароля за валідним зареєстрованим email</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Запит на відновлення пароля за зареєстрованим email</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -754,10 +773,10 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -767,9 +786,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Відображається повідомлення про надсилання інструкцій на вказаний email.</t>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Показано повідомлення про надсилання інструкцій; лист не перевірявся (demo не надсилає пошту).</t>
         </is>
       </c>
     </row>
@@ -789,9 +818,9 @@
           <t>F-20</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Запит на відновлення пароля з неіснуючим email</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Відновлення пароля для неіснуючого облікового запису без розкриття його відсутності</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -806,22 +835,32 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Показано однакове нейтральне повідомлення, система не розкриває відсутність запису.</t>
+          <t>BUG-003</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Показано «This username was not found in the database. Please try again.» — факт відсутності запису розкрито.</t>
         </is>
       </c>
     </row>
@@ -841,9 +880,9 @@
           <t>F-30</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Пошук курсу в каталозі за валідним фрагментом назви</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Пошук курсу в каталозі за фрагментом назви без урахування регістру</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -858,10 +897,10 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -871,9 +910,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>Знайдено відповідний курс без урахування регістру символів.</t>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>09:32</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Знайдено курс «Технології тестування програмного забезпечення»; регістр не впливає.</t>
         </is>
       </c>
     </row>
@@ -893,9 +942,9 @@
           <t>F-30</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Пошук курсу за неіснуючим фрагментом назви</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Пошук курсу за рядком, що не має збігів, із повідомленням про порожній результат</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -910,22 +959,32 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>failed</t>
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>passed</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>BUG-009</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>Текст системного повідомлення при порожній вибірці відрізняється від еталона F-30.</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>09:36</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Порожній результат; показано «Жодного курсу не знайдено».</t>
         </is>
       </c>
     </row>
@@ -942,12 +1001,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>F-40</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Успішне самозарахування студента за точним кодовим словом</t>
+          <t>F-40, GUI-50, BL-70</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Самозарахування студента за точним кодовим словом із присвоєнням ролі «Студент»</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -962,10 +1021,10 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -975,9 +1034,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>Студент успішно приєднався до курсу з роллю 'Студент'.</t>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Зараховано, відкрито курс; у «Учасниках» роль «Студент».</t>
         </is>
       </c>
     </row>
@@ -994,12 +1063,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>F-40, GUI-60</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Спроба самозарахування з невірним кодовим словом</t>
+          <t>F-40, GUI-60, BL-70</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Відхилення самозарахування при кодовому слові з іншим регістром</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1014,22 +1083,32 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>BUG-002</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>Повідомлення про невірне кодове слово відображається у верхньому банері замість підпису під полем.</t>
+          <t>BUG-004</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Помилку показано у верхньому банері, поле з qa-pass-2026 не очищене.</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1125,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>F-50</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Завантаження сторінки курсу та перевірка навігаційної панелі</t>
+          <t>F-50, GUI-75, P-10</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Сторінка курсу: секції, робочий лівий індекс і верхня навігаційна панель</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1066,10 +1145,10 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1079,9 +1158,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Всі розділи курсу та індекс лівої панелі завантажуються коректно.</t>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>5 секцій, робочі посилання індексу, HTTP 200 за 1.2 с (однокористувацький замір).</t>
         </is>
       </c>
     </row>
@@ -1101,9 +1190,9 @@
           <t>F-60, GUI-30</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Здача практичного завдання до дедлайну з файлом .pdf</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Здача завдання файлом report.pdf до дедлайну зі зміною статусу</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1118,10 +1207,10 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1131,9 +1220,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>Статус змінено на 'Здано для оцінювання', файл збережено.</t>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Статус «Здано для оцінювання», дата 21.10.2026 09:57, позначки запізнення немає.</t>
         </is>
       </c>
     </row>
@@ -1150,12 +1249,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>F-60, GUI-30</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Спроба завантаження файлу недозволеного формату (.exe)</t>
+          <t>GUI-30, F-60</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Блокування завантаження файлу .exe у формі здачі завдання</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1170,22 +1269,32 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>BUG-003</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Система дозволила завантажити файл .exe без валідації типу та блокування форми.</t>
+          <t>BUG-005</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>solution.exe прийнято, статус змінився на «Здано для оцінювання».</t>
         </is>
       </c>
     </row>
@@ -1205,9 +1314,9 @@
           <t>GUI-30</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Гранична перевірка розміру файлу (20.00 МБ vs 20.01 МБ)</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Граничний розмір файлу: 20.00 МБ приймається, 20.01 МБ відхиляється</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1222,10 +1331,10 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1235,9 +1344,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Файл 20.00 МБ успішно завантажено, файл 20.01 МБ заблоковано валідатором форми.</t>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>20.00 МБ прийнято, 20.01 МБ відхилено. Дані перестворено після скидання о 10:00.</t>
         </is>
       </c>
     </row>
@@ -1257,9 +1376,9 @@
           <t>GUI-30</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Гранична перевірка кількості файлів (5 шт. vs 6 шт.)</t>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Гранична кількість файлів: 5 приймаються, 6-й блокується</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1274,22 +1393,32 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>failed</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>5 файлів додано успішно, спроба додати 6-й файл заблокована інтерфейсом.</t>
+          <t>BUG-006</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Після 5 файлів 6-й lab1_p6.pdf додано; у списку 6 файлів, збереження успішне.</t>
         </is>
       </c>
     </row>
@@ -1309,9 +1438,9 @@
           <t>F-60, BL-30</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Автоматичне нарахування штрафу 10% за 1 день запізнення</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Штраф 10% за здачу на один день пізніше дедлайну</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1326,22 +1455,32 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>BUG-004</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>У журналі оцінок виставлено 100.00 замість 90.00 балів. Автоштраф 10% не спрацював.</t>
+          <t>BUG-007</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>За роботу, здану на 1 день пізніше, виставлено 100 і зараховано 100.00; штрафу немає.</t>
         </is>
       </c>
     </row>
@@ -1361,9 +1500,9 @@
           <t>F-60, BL-30</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Гранична перевірка максимального порогу штрафу 50% (5 і 6 днів)</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Обмеження штрафу 50% при запізненні на 5 і 6 днів</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1378,22 +1517,32 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>BUG-004</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>Блоковано дефектом BUG-004: оскільки автоштраф не нараховується, перевірити 50% поріг у Web UI неможливо.</t>
+          <t>BUG-007</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>blocked: автоштраф не нараховується взагалі (BUG-007), тому перевірити межу 50% на 5 і 6 днів неможливо.</t>
         </is>
       </c>
     </row>
@@ -1413,9 +1562,9 @@
           <t>F-70</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Оцінювання практичної роботи викладачем з відгуком</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Оцінювання роботи викладачем із балом і текстовим відгуком</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1430,10 +1579,10 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1443,9 +1592,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Оцінка та коментар збережені, відображаються у студента.</t>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Оцінка 95.00 і відгук видимі студенту.</t>
         </is>
       </c>
     </row>
@@ -1462,12 +1621,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>F-80</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Успішне проходження тестування студентом</t>
+          <t>F-80, GUI-40, BL-60</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Проходження тесту з переходом між питаннями та автоматичним підрахунком</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1482,10 +1641,10 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1495,9 +1654,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Відповіді збережені, результат обчислено та відображено на сторінці огляду.</t>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Перехід між питаннями зберігає відповіді; результат 100.00%.</t>
         </is>
       </c>
     </row>
@@ -1517,9 +1686,9 @@
           <t>F-80</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Гранична перевірка ліміту спроб тестування (до 3 спроб)</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Ліміт 3 спроби тесту: четверта спроба недоступна</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1534,22 +1703,32 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>BUG-007</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Після завершення 3 спроб кнопка 'Спроба тесту' залишається активною, дозволено 4-ту спробу.</t>
+          <t>BUG-008</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Після 3 спроб кнопка «Спроба тесту» активна; 4-та спроба починається.</t>
         </is>
       </c>
     </row>
@@ -1569,9 +1748,9 @@
           <t>F-80, BL-40</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Завершення спроби тесту без вибору варіантів</t>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Завершення спроби тесту без жодної відповіді</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1586,10 +1765,10 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1599,9 +1778,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Спроба зарахована з оцінкою 0.0%, система опрацювала стан без помилок.</t>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>10:47</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Порожня спроба зарахована як 0.00 з 2.00 (0.0%).</t>
         </is>
       </c>
     </row>
@@ -1618,12 +1807,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BL-50</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Нарахування часткового балу в тесті з множинним вибором</t>
+          <t>F-80, BL-50</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Частковий бал за питання з кількома правильними відповідями</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1638,10 +1827,10 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1651,9 +1840,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Частковий бал розраховано за формулою без виходу у від'ємні значення.</t>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>За питання з 2 правильними відповідями нараховано 0.50 з 1.00.</t>
         </is>
       </c>
     </row>
@@ -1673,9 +1872,9 @@
           <t>F-90, GUI-80</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Створення нової теми для обговорення на форумі курсу</t>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Створення викладачем нової теми форуму та доступність редагування автором</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1690,10 +1889,10 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Firefox 131 / Win 11</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1703,9 +1902,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Тему опубліковано, редагування автором доступне протягом 30 хвилин.</t>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Тему створено; автору доступне «Редагувати».</t>
         </is>
       </c>
     </row>
@@ -1725,9 +1934,9 @@
           <t>GUI-80</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Спроба створення теми форуму з порожнім полем 'Тема'</t>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Блокування публікації теми форуму з порожнім полем «Тема»</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1742,22 +1951,32 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>failed</t>
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>passed</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>BUG-005</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Текст повідомлення про обов'язкове поле не збігається із затвердженим макетом GUI-80.</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Форма не надіслана; підказка «Заповніть це поле»; теми немає. Дані перестворено після скидання о 11:00.</t>
         </is>
       </c>
     </row>
@@ -1777,9 +1996,9 @@
           <t>F-90</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Автоматичне маркування повідомлення зі стоп-словом</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Маркування повідомлення форуму зі стоп-словом для перевірки викладачем</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1794,22 +2013,32 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>BUG-006</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>Повідомлення зі стоп-словом опубліковано без маркування 'Потребує перевірки' для викладача.</t>
+          <t>BUG-009</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Повідомлення зі словом «спойлер» опубліковано й видиме іншим; маркера «Потребує перевірки» немає.</t>
         </is>
       </c>
     </row>
@@ -1829,9 +2058,9 @@
           <t>F-100, GUI-45</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Перегляд персонального журналу оцінок студентом</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Журнал оцінок студента: стовпці, підсумок і літера ECTS</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1846,10 +2075,10 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -1859,9 +2088,19 @@
           <t>BUG-010</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>У персональному журналі оцінок відсутній обов'язковий стовпець шкали ECTS (A-F).</t>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>У журналі оцінок 7 стовпців без ECTS; підсумок 88.50 без літери.</t>
         </is>
       </c>
     </row>
@@ -1878,12 +2117,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>BL-20</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Гранична верифікація шкали ECTS на стику Fx та E (59.99 vs 60.00)</t>
+          <t>F-100, BL-20</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Межа шкали ECTS Fx/E у журналі оцінок: 59.99 і 60.00</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1898,10 +2137,10 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
@@ -1911,9 +2150,19 @@
           <t>BUG-010</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>Блоковано дефектом BUG-010: відсутність літери ECTS у Web UI унеможливлює перевірку стику 59.99/60.00.</t>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>blocked: стовпця ECTS немає (BUG-010), тому літеру для 59.99 і 60.00 перевірити неможливо.</t>
         </is>
       </c>
     </row>
@@ -1930,12 +2179,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>BL-20</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Гранична верифікація шкали ECTS на стику B та A (94.99 vs 95.00)</t>
+          <t>F-110</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Редагування профілю студента та модерація зміни ПІБ</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1950,10 +2199,10 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Java Module / Contract</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -1963,9 +2212,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>Верифіковано за контрактом класу GradeCalculator.ectsLetter (переноситься в JUnit 5 Спринту 4).</t>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Місто й опис збережено; зміна прізвища — на модерації, старе значення залишилось.</t>
         </is>
       </c>
     </row>
@@ -1982,12 +2241,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>BL-10</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Гранична перевірка суми ваг оцінюваних елементів (99.9% vs 100%)</t>
+          <t>F-120</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Календар: події дедлайнів курсу та створення особистої події</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2002,10 +2261,10 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Java Module / Contract</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
+          <t>Firefox 131.0.3 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -2015,9 +2274,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Верифіковано за контрактом GradeCalculator.weightedTotal (викидає IllegalArgumentException).</t>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Події завдання і тесту відображаються; особисту подію створено.</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2303,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>BL-70, BL-80</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Перевірка блокування зарахування при невиконаному пререквізиті</t>
+          <t>GUI-70, GUI-90</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Адаптивне подання календаря на 375 px і кросбраузерність Chrome/Firefox</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2054,10 +2323,10 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Java Module / Contract</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -2067,9 +2336,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>Верифіковано за контрактом EnrollmentValidator.violations (повертає ERR_PREREQUISITE).</t>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Desktop 1920 px і 375×812: мобільний список, без горизонтальної прокрутки, тач-таргети ≥ 44 px.</t>
         </is>
       </c>
     </row>
@@ -2089,9 +2368,9 @@
           <t>F-130</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Спроба створення курсу менеджером з дублюванням короткої назви</t>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Заборона створення курсу з дубльованою короткою назвою</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2106,10 +2385,10 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Chrome 130 / Win 11</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
+          <t>Chrome 130.0.6723.70 / Windows 11 23H2</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>passed</t>
         </is>
@@ -2119,13 +2398,24 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>Створення заблоковано, виведено повідомлення про те, що коротка назва вже використовується.</t>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Створення заблоковано повідомленням про зайняту коротку назву.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2136,29 +2426,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Параметр тестового середовища</t>
+          <t>Параметр</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значення / Конфігурація</t>
+          <t>Значення</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Рівень / Призначення</t>
+          <t>Призначення</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2170,61 +2460,61 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>URL демонстраційного стенду</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
+          <t>URL demo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>https://sandbox.moodledemo.net</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Веб-сервер / Інтернет</t>
+          <t>Середовище виконання</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Активний, доступний</t>
+          <t>Доступний</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Версія платформи LMS</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Moodle 4.4+ (Build 20261020) / ЕдуПортал v1.1</t>
+          <t>Дата зрізу demo</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>21.10.2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Application Layer</t>
+          <t>Фіксація версії</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Верифіковано</t>
+          <t>Зафіксовано</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Серверна операційна система</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Linux Ubuntu 22.04 LTS (x86_64)</t>
+          <t>Платформа</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Moodle 4.4 (ЕдуПортал v1.1)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Server OS</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2236,105 +2526,105 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Веб-сервер та інтерпретатор</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Apache 2.4.58 / PHP 8.2.18 (OPcache ON)</t>
+          <t>Клієнтська ОС</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Windows 11 Pro 23H2 (22631.4317)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Web / Runtime</t>
+          <t>Робоча станція</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Верифіковано</t>
+          <t>Використовується</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Система керування БД</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>MariaDB 10.11.7 (InnoDB, UTF8mb4)</t>
+          <t>Основний браузер</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 130.0.6723.70 (64-bit)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Web-клієнт</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Верифіковано</t>
+          <t>Використовується</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Клієнтська операційна система</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Microsoft Windows 11 Pro 64-bit (23H2)</t>
+          <t>Другий браузер</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Mozilla Firefox 131.0.3 (64-bit)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Client OS</t>
+          <t>Web-клієнт</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Робоча станція інженера</t>
+          <t>Використовується</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Основний браузер тестування</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Google Chrome 130.0.6723.70 (64-bit)</t>
+          <t>Роздільна здатність</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>1920×1080; емуляція 375×812</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Web Client</t>
+          <t>Desktop / mobile</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Встановлено</t>
+          <t>Використовується</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Вторинний браузер тестування</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Mozilla Firefox 131.0.3 (64-bit)</t>
+          <t>Мова інтерфейсу</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Українська (uk)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Web Client</t>
+          <t>Локалізація</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2346,176 +2636,132 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Роздільна здатність Desktop</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>1920x1080 Full HD (100% DPI, 60 Hz)</t>
+          <t>Акаунт admin</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>admin / sandbox24</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Display</t>
+          <t>Адміністратор</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Стандарт десктоп</t>
+          <t>Перевірено</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Роздільна здатність Mobile</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>375x812 CSS px (Device Emulation: iPhone 13/14)</t>
+          <t>Акаунт manager</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>manager / sandbox24</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Mobile Viewport</t>
+          <t>Менеджер курсів</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Емуляція DevTools</t>
+          <t>Перевірено</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Локалізація інтерфейсу</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Українська мова (uk_UA.utf8 / uk_moodle)</t>
+          <t>Акаунт teacher</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>teacher / sandbox24</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Localization</t>
+          <t>Викладач</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Встановлено за замовчуванням</t>
+          <t>Перевірено</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Тестовий акаунт: Адміністратор</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>admin / sandbox24</t>
+          <t>Акаунт student</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>student / sandbox24</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Site Administrator</t>
+          <t>Студент</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Верифіковано</t>
+          <t>Перевірено</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Тестовий акаунт: Викладач</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>teacher / sandbox24</t>
+          <t>Скидання даних</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Щогодини на початку години</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Teacher (Editing)</t>
+          <t>Обмеження demo</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Верифіковано</t>
+          <t>Враховано; дані перестворено (S7)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Тестовий акаунт: Студент</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>student / sandbox24</t>
+          <t>Модуль Java</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ua.kpi.tzyapz.eduportal</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>BL-вимоги</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Верифіковано</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Тестовий акаунт: Менеджер</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>manager / sandbox24</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Course Manager</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Верифіковано</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Модуль бізнес-логіки Java</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>ua.kpi.tzyapz.eduportal (Java 17, Maven 3.9)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Backend Business Logic</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Готово до Спринту 4</t>
+          <t>У Спринті 3 не виконувався; JUnit 5 у Спринті 4</t>
         </is>
       </c>
     </row>

</xml_diff>